<commit_message>
added DeseasesPage and DeasesPage
</commit_message>
<xml_diff>
--- a/Database/deseases.xlsx
+++ b/Database/deseases.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antipozitife/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antipozitife/Desktop/sealara/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918A5CB6-CF18-6642-8E9B-A00BBD1A8D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FCE16DB-251D-7145-96A8-DEE0FD2B7D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{FFCC9D57-F35F-E246-9B37-28BBBD85C62B}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16100" xr2:uid="{FFCC9D57-F35F-E246-9B37-28BBBD85C62B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="536">
   <si>
     <t>№</t>
   </si>
@@ -3047,12 +3047,21 @@
   <si>
     <t>Глобально (повсеместно) | Восточная Европа и СНГ (Россия, Беларусь, Казахстан) | Северная и Центральная Европа | Северная Америка | Центральная Азия</t>
   </si>
+  <si>
+    <t>картинка</t>
+  </si>
+  <si>
+    <t>https://www.smclinic.ru/upload/iblock/c6f/1uz4ysvcc7q6s5x9wk78mmy7lky1027n.jpg.webp</t>
+  </si>
+  <si>
+    <t>https://www.smclinic.ru/upload/iblock/0a5/1fuyi6hi70ieaao7xb2frk7i9sdpdexk.jpg.webp</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3078,6 +3087,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -3096,10 +3113,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
@@ -3113,14 +3131,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3453,7 +3469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9421AA35-C797-EB48-B98A-18AB923DBDE8}">
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.5" style="1" customWidth="1"/>
@@ -3470,7 +3486,7 @@
     <col min="15" max="15" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="38" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="38" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3516,8 +3532,11 @@
       <c r="O1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>533</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -3563,8 +3582,11 @@
       <c r="O2" s="4" t="s">
         <v>23</v>
       </c>
+      <c r="P2" s="5" t="s">
+        <v>534</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <f>A2 + 1</f>
         <v>2</v>
@@ -3611,8 +3633,11 @@
       <c r="O3" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="P3" s="5" t="s">
+        <v>535</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <f t="shared" ref="A4:A48" si="0">A3 + 1</f>
         <v>3</v>
@@ -3656,11 +3681,11 @@
       <c r="N4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="O4" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -3668,7 +3693,7 @@
       <c r="B5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>83</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -3695,20 +3720,20 @@
       <c r="K5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="O5" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -3716,7 +3741,7 @@
       <c r="B6" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>88</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -3743,20 +3768,20 @@
       <c r="K6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="O6" s="5" t="s">
+      <c r="O6" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -3764,7 +3789,7 @@
       <c r="B7" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="1" t="s">
         <v>93</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -3791,20 +3816,20 @@
       <c r="K7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="O7" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -3812,7 +3837,7 @@
       <c r="B8" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="1" t="s">
         <v>93</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -3839,20 +3864,20 @@
       <c r="K8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="1" t="s">
         <v>84</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O8" s="5" t="s">
+      <c r="O8" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -3860,7 +3885,7 @@
       <c r="B9" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="1" t="s">
         <v>94</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -3887,20 +3912,20 @@
       <c r="K9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="L9" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="O9" s="5" t="s">
+      <c r="O9" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -3908,7 +3933,7 @@
       <c r="B10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -3935,20 +3960,20 @@
       <c r="K10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L10" s="5" t="s">
+      <c r="L10" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M10" s="5" t="s">
+      <c r="M10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="O10" s="5" t="s">
+      <c r="O10" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -3956,7 +3981,7 @@
       <c r="B11" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="1" t="s">
         <v>96</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -3983,20 +4008,20 @@
       <c r="K11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="L11" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="M11" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="N11" s="6" t="s">
+      <c r="N11" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="O11" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -4004,7 +4029,7 @@
       <c r="B12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="1" t="s">
         <v>97</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -4034,17 +4059,17 @@
       <c r="L12" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="M12" s="5" t="s">
+      <c r="M12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="O12" s="5" t="s">
+      <c r="O12" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -4092,7 +4117,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -4140,7 +4165,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -4188,7 +4213,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -5767,6 +5792,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="P2" r:id="rId1" xr:uid="{CF71BBC1-C361-B04C-8EE0-74236E89983D}"/>
+    <hyperlink ref="P3" r:id="rId2" xr:uid="{ED3922B6-7AEF-EB4A-9FCC-7F77BF01BB7E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>